<commit_message>
NMR page: practitioners' practice websites saved live
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/nmr.xlsx
+++ b/downloads/nmr.xlsx
@@ -19,7 +19,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other pages, books and newspape" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other pages, books and newsp 2" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People who endorsed Dr. Levy on" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organizations that sponsored or" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMR practitioners' practice web" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Organizations that sponsored or" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -455,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -661,13 +662,28 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>NMR practitioners' practice web</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>17</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>NMR practitioners' practice websites, saved live on 2026-10-24 (17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
           <t>Organizations that sponsored or</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>13</v>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Organizations that sponsored or hold NMR records</t>
         </is>
@@ -687,6 +703,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId13"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5241,6 +5258,463 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="37" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Pages saved</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Every saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Beeson, Alan</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>beesonchiro.janeapp.com</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>home page</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Begg, Ashton</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>soschiro.net</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Neuromuscular Reeducation Nmr</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bisaccia, John J; Bisaccia, Marna M</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Nmr</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bretow, Steve; Honigman, Ann</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>westside-berkeley-chiropractor.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>About Us; Faq; Our Techniques</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Chesterman, Chris</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>back2best.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Neuromuscular Reeducation</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Ho, Harry</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>elitechirosports.com</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>home page · services · our-team · our-athletes</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Jackson, Gil; Jackson, Stacy</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>gilandstacychiropractic.com</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Article On Nmr; Clinic; Doctor 62518; Home Page</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kane, James</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>summervillespineanddisc.com</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>home page · meet-the-doctor · services-techniques · massage-therapy · about-us</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lane, Eric</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>drericlane.com</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>home page</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Marquis, David</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>pathwaystohealth.net</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Nmr</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Musselman, Bernard</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>bernardmusselman.dr-leonardo.com</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Home Page</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>O'Shaughnessy, Julie</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Contact; Nmr Neuromuscular Reeducation; Therapeutic Soft Tissue Treatment</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Scott, Bridget</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>scottchirodanville.com</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Reviews; What We Do</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Traum, Edward</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>3dintegratedmedical.com</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>home page</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Watson, Amy</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>sweetlightwellness.wordpress.com</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>About</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>practitioner not identified</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>beachcitieschiropractor.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Neuromuscular Re Education</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>practitioner not identified</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>saigechiropractic.com</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Home Page</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId39"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
NMR: certified practitioners in their own words (31 pages), services offered with NMR, template note; new Website examples page (office tours, interactive tools, CV layouts, NFL team chiropractors)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/downloads/nmr.xlsx
+++ b/downloads/nmr.xlsx
@@ -9,16 +9,17 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Index" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Practitioner websites saved" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certified practitioners whose" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key facts" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levy websites and social" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levy YouTube videos" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMR practitioners" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMR website testimonials" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other mentions of NMR" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other mentions of NMR 2" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn endorsers of Levy" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sponsoring organizations" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Certified practitioners in" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What they offer alongside NMR" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key facts" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levy websites and social" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Levy YouTube videos" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMR practitioners" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NMR website testimonials" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other mentions of NMR" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Other mentions of NMR 2" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LinkedIn endorsers of Levy" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sponsoring organizations" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +49,12 @@
       <color rgb="001C458C"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001C458C"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +64,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001C458C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE4F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,11 +84,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -500,116 +511,116 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Certified practitioners whose</t>
+          <t>Certified practitioners in</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Certified practitioners whose websites mention NMR (12)</t>
+          <t>Certified practitioners in their own words: where they discuss NMR (31)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Key facts</t>
+          <t>What they offer alongside NMR</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Key facts, with public sources</t>
+          <t>What they offer alongside NMR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Levy websites and social</t>
+          <t>Key facts</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Dr. Levy's websites and social accounts</t>
+          <t>Key facts, with public sources</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Levy YouTube videos</t>
+          <t>Levy websites and social</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dr. Levy's YouTube videos (34)</t>
+          <t>Dr. Levy's websites and social accounts</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>NMR practitioners</t>
+          <t>Levy YouTube videos</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>NMR practitioners</t>
+          <t>Dr. Levy's YouTube videos (34)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>NMR website testimonials</t>
+          <t>NMR practitioners</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Testimonials on the NMR websites (71)</t>
+          <t>NMR practitioners</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Other mentions of NMR</t>
+          <t>NMR website testimonials</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Other pages, books and newspapers that mention NMR</t>
+          <t>Testimonials on the NMR websites (71)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Other mentions of NMR 2</t>
+          <t>Other mentions of NMR</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -620,28 +631,43 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>LinkedIn endorsers of Levy</t>
+          <t>Other mentions of NMR 2</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>155</v>
+        <v>8</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>People who endorsed Dr. Levy on LinkedIn (155)</t>
+          <t>Other pages, books and newspapers that mention NMR</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>LinkedIn endorsers of Levy</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>155</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>People who endorsed Dr. Levy on LinkedIn (155)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>Sponsoring organizations</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B16" t="n">
         <v>13</v>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Organizations that sponsored or hold NMR records</t>
         </is>
@@ -660,12 +686,513 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>What it is</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Every saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Obituary</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Santa Barbara Independent, 2021-03-04</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>independent.com/obits/2021/03/04/dr-peter-joseph-levy/</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Podcast</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chiropractic Philanthropist ep. 165: Dr. Peter Levy</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>chiropracticphilanthropist.com/165-dr-peter-levy-creating-the-practice</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jackson Chiropractic, Lafayette CA: 'Article on NMR' (Glum developed NMR; Levy handpicked)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>gilandstacychiropractic.com/article%20on%20nmr.html</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Article</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Jackson Chiropractic, Lafayette CA: 'What is NMR'</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>gilandstacychiropractic.com/what%20is%20nmr.html</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Event</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>McTimoney WCCS chapter: Dr Peter Levy NMR seminar</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>mccwccs.weebly.com/events-link/dr-peter-levy-neuromuscular-reeducation</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Yelp: Peter J Levy DC</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>yelp.com/biz/peter-j-levy-dc-santa-barbara-4</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>WebMD</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>doctor.webmd.com/doctor/peter-levy-f195af3f-0ee4-46a3-8558-a7e25166a45</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vitals</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>vitals.com/doctors/Peter_Joseph_Levy.html</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Wellness.com</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>wellness.com/dir/6168598/chiropractor/ca/santa-barbara/peter-levy-dc</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Directory</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ChiroDirectory</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>chirodirectory.com/chiropractors/CA/Santa%20Barbara/Dr-Peter-Levy-0124</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Williston Chiropractic (VT): NMR</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com/treatments/specialized-treatments/nmr/</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Back2Best (Oxford UK): NMR</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>back2best.com/neuromuscular-reeducation/</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Restorative Care Chiropractic (GA): NMR</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com/chiropractic-services/nmr-neuromuscula</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Restorative Care blog: NMR in Peachtree City</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com/blog/understanding-neuromuscular-reedu</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CT Shoreline: Neuro-Muscular Reeducation</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>ctshorelinenutritionresponsetesting.com/Neuro-Muscular-Reeducation</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Wayback</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jeff Banas, Gilbert AZ: Active Release (mentions NMR)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>sportstherapygilbertaz.com/index.php/active-release-gilbert-az/</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Book site</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Dr. Michael Gazdar (Walnut Creek): books</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>gazdar.com/books-by-dr-gazdar/</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Book site</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Dr. Michael Gazdar: about</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>gazdar.com/meet-dr-michael-gazdar/</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Checked, no Levy</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Chiropractic Economics: code 97112 article (2020)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>chiroeco.com/neuromuscular-reeducation/</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>latest saved copy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId38"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -847,7 +1374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4713,7 +5240,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5433,12 +5960,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="65" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5449,239 +5976,809 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>Page that mentions NMR</t>
+          <t>What the page says</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <t>What it says</t>
+          <t>Page</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Bigelow, Brian T</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>bigelowchiropractic.com/services.html</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>se Scoliosis Repatterning Therapeutic Massage Detoxification Vibracussor Instrument Neuromuscular Reeduction Technique (NMR) Infrared Sauna SunLighten Infrared saunas are an effective tool for natural healing and prevention. Infrared light has</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Says they are certified in NMR or trained by Dr. Levy (11)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bisaccia, John J</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>willistonchiropractic.com/</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>s Services/Treatments Conditions treated Common treatments Specialized Treatments Flexion Distraction Graston Technique NMR New Patient Info Insurance Info Articles About Chiropractic Airplane Travel Tips Arthritis Backpack Safety Concussions</t>
+          <t>Craig DeFries, D.C. Well Adjusted, Boulder, CO</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>and whiplash related temporomandibular joint disorders. He then opened his own practice, Precision Chiropractic, in Corpus Christi, TX and was there until 2004. Upon returning to his hometown of Boulder, Colorado, Dr. DeFries began working with the Center for Neuromuscular Reeducation obtaining their certification as well as becoming an instructor. Also, during this time period he completed course work in extremity a</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>welladjusted1.com/about.html (saved 2012)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bisaccia, Marna M</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>willistonchiropractic.com/</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>s Services/Treatments Conditions treated Common treatments Specialized Treatments Flexion Distraction Graston Technique NMR New Patient Info Insurance Info Articles About Chiropractic Airplane Travel Tips Arthritis Backpack Safety Concussions</t>
+          <t>David Hallam Active Chiropractic, Peterborough, UK</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>registered with the GCC). He is a member of the McTimoney Chiropractic Association and a licentiate member of the Royal College of Chiropractors. Other training In 2006, David became the second chiropractor in the UK to be certified as a practitioner of the ‘ Neuromuscular Reeducation ‘ soft tissue technique. David also holds a Diploma in Body Massage and a Certificate in Sports massage. He uses his massage skills to</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>activechiropractic.co.uk/david-hallam/ (saved 2017)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cayer, Jeremy</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>healtouchchiro.com/dr-jeremy-cayer/</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>is doctorate, Dr. Cayer has a certification in sports science and human performance, and has advanced certifications in neuromuscular reeducation. In Maryland, he’s also considered a physical therapist and has a stamp on his license indicating he’s a physical</t>
+          <t>Diane Miller Listening Wellness Center, MA</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Connecticut Center for Massage Therapy in Newington, CT. Diane is certified in Pregnancy Massage, Pediatric Massage and Neuro Muscular Re-education. She received her certification in Pregnancy Massage from Elaine Stillerman, LMT. Elaine is the author of Prenatal M</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>listeningwellness.org/portfolio_page/diane-miller/ (saved 2024)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Duckett, Stacey</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>primespineplus.com/</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>body. It is effective in increasing circulation and lymphatic flow with a decrease in muscle spasm. She is certified in Neuro-Muscular Re-education which locates adhesions and releases soft tissue restrictions of the muscles and tendons that helps improve prop</t>
+          <t>Eric Lane, D.C. Tucson Lane Family Chiropractic, Tucson, AZ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Dr. Lane is an avid advocate of Nutrition, Exercise and implements these in his practice. He is a graduate from Parker College of Chiropractic in Dallas Texas. He is Nationally Board Certified. He is also is licensed in Physiotherapy. Dr. Lane is Certified in Neuromuscular Reeducation and Chiropractic BioPhysics. We are committed to you our patients to deliver the best care you deserve. Tucson Lane Family Chiropracti</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>drericlane.com/about_us.html (saved 2011)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hallam, David</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>activechiropractic.co.uk/david-hallam/</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>tion. Other training In 2006, David became the second chiropractor in the UK to be certified as a practitioner of the ‘ Neuromuscular Reeducation ‘ soft tissue technique. David also holds a Diploma in Body Massage and a Certificate in Sports massage. He uses h</t>
+          <t>Eric Lane, D.C. Tucson Lane Family Chiropractic, Tucson, AZ</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PRACTOR SERVICES Return To Services We are pleased to have this wonderful therapy available in our office. Dr. Lane has attained the highest level of certification having been taught and certified by Peter Levy. You may ask what is Neuromuscular Reeducation ? Neuromuscular Reeducationsm is a "stand-alone" hands-on technique/approach to the evaluation and functional treatment of 90+% of the soft tissue injuries a prof</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>drericlane.com/Neuromuscular.html (saved 2011)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Johnson, Jeffrey</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>truchiropractors.com/tru-holistic-injury-recovery</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Soft Tissue Therapy: We utilize a dynamic, non-invasive deep tissue technique known as Neuromuscular Reeducation (NMR)</t>
+          <t>Garry Bracken, D.C. The Sports Therapy Center, Portland, ME</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>h Goulding Chiropractic, Portland,ME. Dr. Garry's post graduate training has focused on Neurology Diplomate studies, Sports Injuries, and various Neuromuscular, deep tissue and Physical Therapy protocals and treatment. Dr. Garry is a Certified Practicioner of Neuromuscular Reeducation http://www.nmrseminars.com/ Dr. Garry is also a Certified Graston Technique Provider http://grastontechnique.com/grastontechnique/defa</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>thesportstherapycenter.com/5.html (saved 2012)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Miller, Diane</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>listeningwellness.org/portfolio_page/diane-miller/ (saved copy)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Connecticut Center for Massage Therapy in Newington, CT. Diane is certified in Pregnancy Massage, Pediatric Massage and Neuro Muscular Re-education. She received her certification in Pregnancy Massage from Elaine Stillerman, LMT. Elaine is the author of Prenat</t>
+          <t>Jeremy Cayer, D.C. Healing Touch Chiropractic</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>is doctorate, Dr. Cayer has a certification in sports science and human performance, and has advanced certifications in neuromuscular reeducation. In Maryland, he’s also considered a physical therapist and has a stamp on his license indicating he’s a physical th</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>healtouchchiro.com/dr-jeremy-cayer/</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mott, Lisa</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>magicmott.com/massage</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Swedish, Deep Tissue, Myofascial Release, Shiatsu, Thai, Orthopedic Massage, Orthopedic Sports Massage, Neurolymphatic, NeuroMuscular Re-education, ART, and NKT are expertly used to give you " the best massage you've ever had! " Initial Visit including Assessm</t>
+          <t>John and Marna Bisaccia, D.C. Williston Chiropractic &amp; Sportsmedicine, Williston, VT</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ngth and Conditioning Association. He received the Vermont Chiropractor of the Year Award in 2007 and VCA’s Distinguished Service Award in 2013. Marna Bisaccia, DC acts as the clinic supervisor. She also specializes in soft tissue problems and is certified in Neuromuscular Reeducation and as a Graston practitioner . Dr. Marna is also certified in Dry Needling. Dr. Marna received a Bachelor’s degree in Business Admini</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com/about/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Poane, Robert</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>drpoane.com/techniques</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>n, muscle tension, hypersensitivity, burning sensations, numbness, tingling and coldness in hands, feet, nose and ears. NMR (Myofascial/Medical Massage) Your myofascial tissue is a network of tissue that spreads throughout your entire body. It</t>
+          <t>Julie O'Shaughnessy, D.C. Restorative Care Chiropractic, Peachtree City, GA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ned to address muscular and joint dysfunction. Originally developed by Dr. Gary Glum and Dr. Joseph Hourigan, this method was further refined and extensively taught by the late Dr. Peter Levy, from whom I had the privilege of learning directly. As a certified NMR practitioner, I've successfully integrated this effective method into my chiropractic practice, uniquely blending it with my background in myofascial releas</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com/blog/understanding-neur (saved 2025)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Townshend, Judith</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>directory.coventrytelegraph.net/company/974755986079744</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>ithtownshend.co.uk Website: Visit Website Message now judith.townshend @judithtownshend chiropractic , sports massage , neuromuscular reeducation , McTimoney chiropractic Report a problem with this listing Business Profile Judith Townshend, Chiroprator Judith</t>
+          <t>Nicole Zollinger-Muench Carmel, IN</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ate practice in Carmel. In her career, she is currently the only person in Indiana who has a specialty certification in Neuromuscular Reeducation (NMR). She has achieved Associate Member Status in the Practitioner Training Program through the Society of Ortho–Bi</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>massagebook.com/Carmel~Massage~nicole-zollinger-muench</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Zollinger-Muench, Nicole</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>massagebook.com/Carmel~Massage~nicole-zollinger-muench</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>ate practice in Carmel. In her career, she is currently the only person in Indiana who has a specialty certification in Neuromuscular Reeducation (NMR). She has achieved Associate Member Status in the Practitioner Training Program through the Society of Ortho–</t>
+          <t>Stacey Duckett, D.C. Prime Spine Plus, Antioch, CA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>body. It is effective in increasing circulation and lymphatic flow with a decrease in muscle spasm. She is certified in Neuro-Muscular Re-education which locates adhesions and releases soft tissue restrictions of the muscles and tendons that helps improve proper m</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>primespineplus.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Explains how NMR works (8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Derek Taylor, D.C. Taylor Chiropractic &amp; Laser Center, Torrance, CA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>: "¢ T he Gonstead T echnique "¢ Nimmo Receptor Tonus Technique (Travel Myofascial Release) "¢ Graston Technique "¢ Body Restoration Technique "¢ Biocranial Therapy "¢ Reflex Nutrition Assessment "¢ Gonzalez Rehab Technique "¢ Matrix re-patterning "¢ Neuromuscular Reeducation technique "¢ Brimhall Technique "¢ Dynamic Joint Recovery "¢ Class IV Avicenna Laser "¢ K-Laser Dr. Taylor &gt;&gt; Our Office &gt;&gt; login:</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>drderektaylor.com/about/torrance-chiropractic.html (saved 2011)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Gil and Stacy Jackson Jackson Chiropractic, Lafayette, CA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ng in between. Muscles are links in a chain of joints; they act together and are apt to suffer together; this is especially true of muscles on the sound side of the body which have a tendency to overwork. "'The key to understanding the technique I use, called Neuromuscular Re-education, is knowing about adhesions,' Levy said. All of a sudden the light bulb flashed on: This was the doctor that Dr. Gary Glum, co-founde</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>gilandstacychiropractic.com/what%20is%20nmr.html (saved 2011)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>John Hayes, D.C. (Hayes Chiropractic Center) Portland, ME</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ed by a fibrous healing, and the laying down of elastic (poorly vascularized scar tissue) to protect the involved areas. These are further known as adhesions and occur wherever damage and inflammation have occurred, limiting both strength and range of motion. NMR locates these adhesions that are specifically related to abnormal motion and due to old trauma. By applying deep and, what some may consider painful, pressu</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>hayeschiropracticcenter.com/services/neuromuscularreedu (saved 2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Julie O'Shaughnessy, D.C. Restorative Care Chiropractic, Peachtree City, GA</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>from patients is that they have lived with this pain for a long enough period of time that any pain as a result of treatment is not a big concern if it will help resolve the problem. 2. How long does the therapy take to work? In all reality the application of neuromuscular reeducation should show a definitive change in range of motion, function, and possibly pain almost immediately. When running a clinical trial on a</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com/chiropractic-services/n (saved 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lisa Mott Magic Mott massage</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Swedish, Deep Tissue, Myofascial Release, Shiatsu, Thai, Orthopedic Massage, Orthopedic Sports Massage, Neurolymphatic, NeuroMuscular Re-education, ART, and NKT are expertly used to give you " the best massage you've ever had! " Initial Visit including Assessment</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>magicmott.com/massage</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Robert Poane, D.C. Dr. Poane, CT</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>d sensitivity symptoms. Visit Our Office Today Injuries Automobile Accident Worker’s Compensation Sports Recreational Techniques Diversified Method of manipulation Activator Method of manipulation Sacro Occipital Techniques Special Table for Pregnant Patients NMR (myofascial / medical massage) Emotional Freedom Technique (EFT) Ionic Foot Bath Neurologic Stress Reduction Therapy (NSRT) Advanced Allergy Therapeutics (A</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>drpoane.com/ (saved 2016)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Robert Poane, D.C. Dr. Poane, CT</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>n, muscle tension, hypersensitivity, burning sensations, numbness, tingling and coldness in hands, feet, nose and ears. NMR (Myofascial/Medical Massage) Your myofascial tissue is a network of tissue that spreads throughout your entire body. It</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>drpoane.com/techniques</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Westside Family Chiropractic Berkeley, CA</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>the table to assist the adjustment. Individual cushions or "drop pieces" located along the table support each area of the spine until the thrust is given. Then, each drop-piece gently gives way, reducing the pressure needed to move a specific spinal segment. Neuro Muscular Reeducation Technique This is a precursor to Active Release Technique. This is a new and highly successful approach to injuries This is a precurso</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>westside-berkeley-chiropractor.com/our-techniques/ (saved 2012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Lists NMR among the services offered (10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Brian T. Bigelow, D.C. Bigelow Chiropractic Center, Nashua, NH</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bigelow Chiropractic Center Favorite Websites: www.teamintraining.org www.nmrseminars.com Anthrostim 1 Dear Mr. Miller, i recently had the opportunity to be treated with download Anthrostim 2 Chiropractic adjustments helps stimulate the body to heal itself. download Interactive Spine Click Here The chiropractic science was developed in 1895 and has since become the fastest growing primary healthcare pr</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>bigelowchiropractic.com:80/ (saved 2006)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Brian T. Bigelow, D.C. Bigelow Chiropractic Center, Nashua, NH</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>se Scoliosis Repatterning Therapeutic Massage Detoxification Vibracussor Instrument Neuromuscular Reeduction Technique (NMR) Infrared Sauna SunLighten Infrared saunas are an effective tool for natural healing and prevention. Infrared light has</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>bigelowchiropractic.com/services.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Connie Grantham, D.C. Crawford Family Chiropractic, CO</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>My specialty lies in helping those suffering from soft-tissue injury. Professional Therapy Services: Craniosacral Kinesio Taping McKenzie Technique Gua Sa Certified Functional Medicine Practioner Mulligan Practioner Myofacial Release and Viseral manipulation Neuromuscular Re-education Therapeutic and Functional Exercise I provide chiropractic care for the whole family in a warm and safe home environment. I use a wide</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>crawfordfamilychiro.com/services (saved 2020)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Darryl Koch, D.C. Community Chiropractic Spine and Sport, Essex Junction, VT</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>for seven years. Dr. Koch received his Chiropractic Sports Physician certicfication (CCSP) in 1998. He has updated his technique and knowledge base by attending numerous continuing education seminars including upper cervical techniques, functional neurology, Neuro-Muscular Reeducation (NMR), work place ergonomics, whiplash and sports injuries. An active member of the Vermont Chiropractic Association, Darryl has serve</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>spineandsportvt.com/about (saved 2012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Darryl Koch, D.C. Community Chiropractic Spine and Sport, Essex Junction, VT</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ies Wrist injuries Hand injuries Upper Leg injuries Knee injuries Lower Leg injuries Ankle injuries Foot injuries Chiropractic care for sports injuries can put you back in the game, and help you avoid further injury. Treatment may include deep tissue massage (NMR), spinal manipulation and physio-therapy modalieties (ice, electrical muscle stimulation &amp; ultrasound). COMMUNITY CHIROPRACTIC SPINE AND SPORT 69 CENTER ROA</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>spineandsportvt.com/sports-injuries (saved 2012)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Jeffrey S. Johnson, D.C. TRUchiropractors, Walnut Creek, CA</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Soft Tissue Therapy: We utilize a dynamic, non-invasive deep tissue technique known as Neuromuscular Reeducation (NMR)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>truchiropractors.com/tru-holistic-injury-recovery (saved 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>John Hayes, D.C. (Hayes Chiropractic Center) Portland, ME</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>tures – nerves, ligaments, tendons and muscles, conditions such as sprains, strains, herniated discs, disc problems, sciatica, headaches, etc. Explore the links to the right or below to see what Hayes Chiropractic Center has to offer! Chiropractic Orthopedics Neuromuscular Reeducation Spinal Manipulative and Soft Tissue Therapies Activator Protocol Graston Technique Impulse Adjustor Supplements and Supports Nutrition</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>hayeschiropracticcenter.com/services1 (saved 2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>John and Marna Bisaccia, D.C. Williston Chiropractic &amp; Sportsmedicine, Williston, VT</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>s Services/Treatments Conditions treated Common treatments Specialized Treatments Flexion Distraction Graston Technique NMR New Patient Info Insurance Info Articles About Chiropractic Airplane Travel Tips Arthritis Backpack Safety Concussions</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Julie O'Shaughnessy, D.C. Restorative Care Chiropractic, Peachtree City, GA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>OK NOW About Policies &amp; Fees Conditions Ankle &amp; Foot Pain Arthritis Back &amp; Neck Pain Carpal Tunnel Syndrome &amp; Wrist Pain Concussions Headaches Hip Pain more... Chiropractic Services Chiropractic Care Prenatal, Infant &amp; Child Chiropractic Care Kinesiology Tape NMR - Neuromuscular Reeducation MPS - Microcurrent Point Stimulation for Pain Relief &amp; Scar Therapy MPS - C-Section Scar Therapy Shockwave Therapy Office: 111 P</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>restorativecarechiropractic.com/about (saved 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>directory.coventrytelegraph.net</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ithtownshend.co.uk Website: Visit Website Message now judith.townshend @judithtownshend chiropractic , sports massage , neuromuscular reeducation , McTimoney chiropractic Report a problem with this listing Business Profile Judith Townshend, Chiroprator Judith is</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>directory.coventrytelegraph.net/company/974755986079744</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Uses "neuromuscular re-education" in the general rehab sense, not Dr. Levy's NMR (2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Josh Duplessis, D.C. Core 1 Chiropractic, Downers Grove, IL</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>orrect posture, we are able to stimulate the nerve signals ensuring they are retrained for appropriate, correct muscle motion. Neuromuscular re-education will be paired with other treatments and therapies to facilitate the restoration of normal movements. The neuromuscular re-education program focuses on restructuring the way the brain and spinal cord react in voluntary and reflexive movement. By retraining the neuro</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>core1chiro.com/neuromuscular-re-education/ (saved 2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Tampa Holistic Chiropractic Tampa, FL</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>auma, medical conditions, and neurological conditions, such as stroke and traumatic brain injury. Neuromuscular re-education is one method used by rehabilitation therapists to facilitate the return of normal movement in persons with neuromuscular impairments. Neuromuscular re-education and movement training is somewhat related to core training. These approaches can be used for patients with spine-related symptoms, or</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>tampaholisticchiro.com/neuromuscular-re-education/ (saved 2021)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Services listed with NMR</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Page</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>John and Marna Bisaccia, D.C. Williston Chiropractic &amp; Sportsmedicine, Williston, VT</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Flexion Distraction · Graston Technique · NMR</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>willistonchiropractic.com/about/</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Julie O'Shaughnessy, D.C. Restorative Care Chiropractic, Peachtree City, GA</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Chiropractic Care · Prenatal, Infant &amp; Child Chiropractic Care · Kinesiology Tape · NMR - Neuromuscular Reeducation · MPS - Microcurrent Point Stimulation for Pain Relief &amp; Scar Therapy · MPS - C-Section Scar Therapy · Shockwave Therapy</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20250428215229/https://re</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>John Hayes, D.C. (Hayes Chiropractic Center) Portland, ME</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Chiropractic Orthopedics · Neuromuscular Reeducation · Spinal Manipulative and Soft Tissue Specialties Activator Protocol · Graston · Impulse Adjuster</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20230328214131/http://www</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Robert Poane, D.C. Dr. Poane, CT</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Diversified Method of manipulation · Activator Method of manipulation · Sacro Occipital Techniques · Special Table for Pregnant Patients · NMR (myofascial / medical massage) · Emotional Freedom Technique (EFT) · Ionic Foot Bath · Neurologic Stress Reduction Therapy (NSRT) · Advanced Allergy Therapeutics (Allergy / sensitivity symptoms)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20160312002851/http://drp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Westside Family Chiropractic Berkeley, CA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Impulse · Drop Table · Neuro Muscular Reeducation Technique</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20120221203246/http://www</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Brian T. Bigelow, D.C. Bigelow Chiropractic Center, Nashua, NH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Nutritional Counselling · Orthotics · Pain Desensitization · Pelvic Blocking · Scar Tissue Release · Scoliosis Repatterning · Therapeutic Massage · Detoxification · Vibracussor Instrument · Neuromuscular Reeduction Technique (NMR)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>bigelowchiropractic.com/services.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Connie Grantham, D.C. Crawford Family Chiropractic, CO</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Mulligan Practioner · Myofacial Release and Viseral manipulation · Neuromuscular Re-education · Therapeutic and Functional Exercise</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20200809133119/https://cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Josh Duplessis, D.C. Core 1 Chiropractic, Downers Grove, IL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Golf Performance · Chiropractic Adjustment · Neuromuscular Re-education · Nutrition Consultation · Muscle Energy Techniques · Postural Training · Manual Therapy · Gait Analysis · Athletic Performance · Acute/ Chronic Pain Management · Orthopedic Assessment · Sport Taping · Exercise Rx</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20211224045315/https://co</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tampa Holistic Chiropractic Tampa, FL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cox Technic · Webster Technique · Pediatric Chiropractic · IQ Impulse · Laser Therapy · Massage Therapy · Hydrotherapy · Rehabilitation Exercise · Heat and Cold Therapy · Electrical Muscle Stimulation · Neuromuscular Re-education · Ultrasound</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>web.archive.org/web/20210416024609/https://ta</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5755,7 +6852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6255,7 +7352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6905,7 +8002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -8444,7 +9541,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11069,504 +12166,4 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
-    <col width="72" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>What it is</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Every saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Obituary</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Santa Barbara Independent, 2021-03-04</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>independent.com/obits/2021/03/04/dr-peter-joseph-levy/</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Podcast</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Chiropractic Philanthropist ep. 165: Dr. Peter Levy</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>chiropracticphilanthropist.com/165-dr-peter-levy-creating-the-practice</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Article</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Jackson Chiropractic, Lafayette CA: 'Article on NMR' (Glum developed NMR; Levy handpicked)</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>gilandstacychiropractic.com/article%20on%20nmr.html</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Article</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Jackson Chiropractic, Lafayette CA: 'What is NMR'</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>gilandstacychiropractic.com/what%20is%20nmr.html</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Event</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>McTimoney WCCS chapter: Dr Peter Levy NMR seminar</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>mccwccs.weebly.com/events-link/dr-peter-levy-neuromuscular-reeducation</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Directory</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Yelp: Peter J Levy DC</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>yelp.com/biz/peter-j-levy-dc-santa-barbara-4</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Directory</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>WebMD</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>doctor.webmd.com/doctor/peter-levy-f195af3f-0ee4-46a3-8558-a7e25166a45</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Directory</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Vitals</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>vitals.com/doctors/Peter_Joseph_Levy.html</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Directory</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Wellness.com</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>wellness.com/dir/6168598/chiropractor/ca/santa-barbara/peter-levy-dc</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Directory</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ChiroDirectory</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>chirodirectory.com/chiropractors/CA/Santa%20Barbara/Dr-Peter-Levy-0124</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Williston Chiropractic (VT): NMR</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>willistonchiropractic.com/treatments/specialized-treatments/nmr/</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Back2Best (Oxford UK): NMR</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>back2best.com/neuromuscular-reeducation/</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Restorative Care Chiropractic (GA): NMR</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>restorativecarechiropractic.com/chiropractic-services/nmr-neuromuscula</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Restorative Care blog: NMR in Peachtree City</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>restorativecarechiropractic.com/blog/understanding-neuromuscular-reedu</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>CT Shoreline: Neuro-Muscular Reeducation</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>ctshorelinenutritionresponsetesting.com/Neuro-Muscular-Reeducation</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Wayback</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Jeff Banas, Gilbert AZ: Active Release (mentions NMR)</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>sportstherapygilbertaz.com/index.php/active-release-gilbert-az/</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Book site</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Dr. Michael Gazdar (Walnut Creek): books</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>gazdar.com/books-by-dr-gazdar/</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Book site</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Dr. Michael Gazdar: about</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>gazdar.com/meet-dr-michael-gazdar/</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Checked, no Levy</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Chiropractic Economics: code 97112 article (2020)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>chiroeco.com/neuromuscular-reeducation/</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>latest saved copy</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId38"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>